<commit_message>
Add Task 5 DistilBERT fine-tuning and shared evaluation helpers. Extract evaluation utilities to src/evaluation.py, refactor Task 3 to use them, and log transformer results in the experiment sheet and report.
</commit_message>
<xml_diff>
--- a/ExperimentSummarySheet_Ex1.xlsx
+++ b/ExperimentSummarySheet_Ex1.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25.42" customWidth="1" style="2" min="1" max="1"/>
@@ -530,410 +530,512 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Naive Bayes</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>BoW</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>multiclass</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>MultinomialNB (default alpha=1.0)</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="2" t="n">
         <v>0.7113</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="2" t="n">
         <v>0.6339</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Many positive→neutral errors; negative recall 0.47.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>figures/naive_bayes_bow_multiclass_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Feed-forward NN</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BoW</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>multiclass</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>MLPClassifier hidden=(128,64), max_iter=300, early_stopping=True, random_state=42</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>0.733</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>0.6693</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Best multiclass macro F1; still confuses positive with neutral.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>figures/feed_forward_nn_bow_multiclass_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Naive Bayes</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>TF-IDF</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>multiclass</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>MultinomialNB (default alpha=1.0)</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="2" t="n">
         <v>0.6763</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="2" t="n">
         <v>0.4184</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>TF-IDF down-weights frequent words; model collapses toward neutral (negative recall 0.01).</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>figures/naive_bayes_tfidf_multiclass_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Feed-forward NN</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>TF-IDF</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>multiclass</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>MLPClassifier hidden=(128,64), max_iter=300, early_stopping=True, random_state=42</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="2" t="n">
         <v>0.7268</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="2" t="n">
         <v>0.6536</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Better than TF-IDF NB; neutral class still dominates predictions.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>figures/feed_forward_nn_tfidf_multiclass_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Naive Bayes</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BoW</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>binary (no neutral)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>MultinomialNB (default alpha=1.0)</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="2" t="n">
         <v>0.8274</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="2" t="n">
         <v>0.7953</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Best overall classical run; subtle positives still misclassified.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>figures/naive_bayes_bow_binary_no_neutral_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Feed-forward NN</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BoW</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>binary (no neutral)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>MLPClassifier hidden=(128,64), max_iter=300, early_stopping=True, random_state=42</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="2" t="n">
         <v>0.8223</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="2" t="n">
         <v>0.7805</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Similar to NB BoW; positive recall higher than negative.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>figures/feed_forward_nn_bow_binary_no_neutral_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Naive Bayes</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>TF-IDF</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>binary (no neutral)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>MultinomialNB (default alpha=1.0)</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="2" t="n">
         <v>0.7386</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="2" t="n">
         <v>0.5647</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>TF-IDF NB again under-detects negative class (recall 0.17).</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>figures/naive_bayes_tfidf_binary_no_neutral_confusion_matrix.png</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Hatice Kubra Aksu / Ray</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Feed-forward NN</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>TF-IDF</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>lowercase, NLTK word_tokenize, English stopword removal</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>binary (no neutral)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>MLPClassifier hidden=(128,64), max_iter=300, early_stopping=True, random_state=42</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="2" t="n">
         <v>0.8198</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="2" t="n">
         <v>0.7729</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>NN handles TF-IDF better than NB in binary setting.</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>figures/feed_forward_nn_tfidf_binary_no_neutral_confusion_matrix.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Hatice Kubra Aksu / Ray</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DistilBERT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>transformer embeddings</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>raw text (no Task 2 preprocessing)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>multiclass</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased, lr=2e-5, batch=16, epochs=3, max_length=128; local Apple Silicon; multiclass ~3.5 min</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.8361</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.8241000000000001</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Best overall model; fewer positive→neutral errors than classical baselines.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>figures/distilbert_multiclass_confusion_matrix.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Hatice Kubra Aksu / Ray</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>DistilBERT</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>transformer embeddings</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>raw text (no Task 2 preprocessing)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>binary (no neutral)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased, lr=2e-5, batch=16, epochs=3, max_length=128; local Apple Silicon; binary ~1.4 min</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.9569</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Strong binary performance; 17 errors on test set.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>figures/distilbert_binary_confusion_matrix.png</t>
         </is>
       </c>
     </row>

</xml_diff>